<commit_message>
Align sig figs of OCCF variables
</commit_message>
<xml_diff>
--- a/InputData/web-app/OCCF/Output Currency Conversion Factors.xlsx
+++ b/InputData/web-app/OCCF/Output Currency Conversion Factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\web-app\OCCF\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\web-app\OCCF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10BBDDCD-D2F2-4949-A193-F5473D591A3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D9F31BD-4707-4779-A701-14F7AA388F50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="58335" yWindow="1830" windowWidth="26355" windowHeight="13080" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -127,6 +127,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="2">
+    <numFmt numFmtId="166" formatCode="0.000000"/>
+    <numFmt numFmtId="169" formatCode="0.00000E+00"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -170,16 +174,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -485,27 +490,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="2" max="2" width="26.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -513,80 +518,80 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="5"/>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="4"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="5"/>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="4"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="5"/>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B23" s="4"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>0.73191600598044548</v>
       </c>
@@ -594,32 +599,32 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B29" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B30" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B31" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B32" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B33" t="s">
         <v>19</v>
       </c>
@@ -636,21 +641,21 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="7">
         <f>10^9*About!$A$26</f>
         <v>731916005.9804455</v>
       </c>
@@ -666,21 +671,21 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="5">
         <f>10^6*About!$A$26</f>
         <v>731916.00598044554</v>
       </c>
@@ -696,21 +701,21 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="2" max="2" width="31.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="B1" s="3" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="B1" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="6">
         <f>1*About!A26</f>
         <v>0.73191600598044548</v>
       </c>

</xml_diff>